<commit_message>
Estimación con dato del 2026-10-05
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -24,6 +24,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-06</t>
   </si>
 </sst>
 </file>
@@ -374,6 +377,17 @@
         <v>0.0198484938629934</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.000378721620414171</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.019460771321152</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-06
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -27,6 +27,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-07</t>
   </si>
 </sst>
 </file>
@@ -388,6 +391,17 @@
         <v>0.019460771321152</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.000381579146888121</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0195340509594943</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-07
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -30,6 +30,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08</t>
   </si>
 </sst>
 </file>
@@ -402,6 +405,17 @@
         <v>0.0195340509594943</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.000377157439338417</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0194205416849896</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-08
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -33,6 +33,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-09</t>
   </si>
 </sst>
 </file>
@@ -416,6 +419,17 @@
         <v>0.0194205416849896</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.000374966388016218</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.0193640488538998</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-09
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -36,6 +36,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-12</t>
   </si>
 </sst>
 </file>
@@ -430,6 +433,17 @@
         <v>0.0193640488538998</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.000425756245306434</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0206338616188641</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-12
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -39,6 +39,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13</t>
   </si>
 </sst>
 </file>
@@ -444,6 +447,17 @@
         <v>0.0206338616188641</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.00041887610439925</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0204664629186201</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-13
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -42,6 +42,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-14</t>
   </si>
 </sst>
 </file>
@@ -458,6 +461,17 @@
         <v>0.0204664629186201</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.000421260445170983</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0205246302078986</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-14
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-15</t>
   </si>
 </sst>
 </file>
@@ -472,6 +475,17 @@
         <v>0.0205246302078986</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.000429938113666646</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0207349490876309</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-15
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -48,6 +48,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-16</t>
   </si>
 </sst>
 </file>
@@ -486,6 +489,17 @@
         <v>0.0207349490876309</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.000430381152020983</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0207456297089527</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-16
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-19</t>
   </si>
 </sst>
 </file>
@@ -500,6 +503,17 @@
         <v>0.0207456297089527</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.000432035249570207</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.020785457646398</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-19
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-20</t>
   </si>
 </sst>
 </file>
@@ -514,6 +517,17 @@
         <v>0.020785457646398</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.000344560114773941</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.0185623305318578</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-20
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-21</t>
   </si>
 </sst>
 </file>
@@ -528,6 +531,17 @@
         <v>0.0185623305318578</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.000348349739299568</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.0186641297493231</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-21
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-22</t>
   </si>
 </sst>
 </file>
@@ -542,6 +545,17 @@
         <v>0.0186641297493231</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.00034960771736895</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.0186977998002158</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-22
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-23</t>
   </si>
 </sst>
 </file>
@@ -556,6 +559,17 @@
         <v>0.0186977998002158</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.000410872141423898</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.020269981288198</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-23
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-26</t>
   </si>
 </sst>
 </file>
@@ -570,6 +573,17 @@
         <v>0.020269981288198</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.00040972173074405</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.0202415841955132</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-26
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-27</t>
   </si>
 </sst>
 </file>
@@ -584,6 +587,17 @@
         <v>0.0202415841955132</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.000406597729759403</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.0201642686393383</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-27
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-28</t>
   </si>
 </sst>
 </file>
@@ -598,6 +601,17 @@
         <v>0.0201642686393383</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.000416411794627985</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.0204061705037468</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-28
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -75,6 +75,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-29</t>
   </si>
 </sst>
 </file>
@@ -612,6 +615,17 @@
         <v>0.0204061705037468</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.000373414217239282</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.0193239286181481</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Estimación con dato del 2026-10-29
</commit_message>
<xml_diff>
--- a/varianza_estimada.xlsx
+++ b/varianza_estimada.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t xml:space="preserve">fecha</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-30</t>
   </si>
 </sst>
 </file>
@@ -626,6 +629,17 @@
         <v>0.0193239286181481</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.000372966827174017</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.0193123490848218</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>